<commit_message>
Regenerate business_results.xlsx with fresh cell-by-cell write
Recreated to fix potential empty-content issue in Gmail attachment.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCNeWRJCWXyKVt3Q81DWqb
</commit_message>
<xml_diff>
--- a/business_results.xlsx
+++ b/business_results.xlsx
@@ -425,13 +425,13 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Update business_results.xlsx with clean no-formatting output
Recreated Excel file using plain ws.append() calls only (no Font,
Alignment, or RTL settings) to ensure valid base64 encoding for
Gmail attachment. Contains finding: ברקוב דניאל - רופאי שיניים
at אבא אחימאיר 205, ירושלים.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCNeWRJCWXyKVt3Q81DWqb
</commit_message>
<xml_diff>
--- a/business_results.xlsx
+++ b/business_results.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="תוצאות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,14 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,85 +415,76 @@
   </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>שם העסק</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>כתובת</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>סוג עסק</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>דירוג אינדיקציה</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>קישור 1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>קישור 2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>קישור 3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ברקוב דניאל - רופאי שיניים</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>אבא אחימאיר 205, ירושלים</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>רופא שיניים</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>https://www.dunsguide.co.il/C2fca8c3525b02805163b104c94ce17ed_%D7%A8%D7%95%D7%A4%D7%90%D7%99_%D7%A9%D7%99%D7%A0%D7%99%D7%99%D7%9D/%D7%91%D7%A8%D7%A7%D7%95%D7%91_%D7%93%D7%A0%D7%99%D7%90%D7%9C</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://www.dunsguide.co.il/L99995816-A5-A5_%D7%A8%D7%95%D7%A4%D7%90%D7%99_%D7%A9%D7%99%D7%A0%D7%99%D7%99%D7%9D/%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D_%D7%95%D7%94%D7%A1%D7%91%D7%99%D7%91%D7%94/%D7%99%D7%A8%D7%95%D7%A9%D7%9C%D7%99%D7%9D_%D7%95%D7%94%D7%A1%D7%91%D7%99%D7%91%D7%94</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>